<commit_message>
Remove temporary Excel file ~$EsitiTest.xlsx
</commit_message>
<xml_diff>
--- a/EsitiTest.xlsx
+++ b/EsitiTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Doc\File python\Finanza\Certificates\Revisione2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5C268E3-32A3-4D82-AF12-EED001FBC83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF7D841-B94B-4CA4-AEFA-2C524036671F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{14AA7898-9A2E-47D6-ACA7-BF325A77C1C7}"/>
   </bookViews>
@@ -483,7 +483,7 @@
   <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
-    <col min="2" max="2" width="40.36328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="48" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.08984375" style="1" customWidth="1"/>
     <col min="4" max="4" width="13.26953125" style="1" customWidth="1"/>
     <col min="5" max="5" width="8.7265625" style="1"/>

</xml_diff>